<commit_message>
completed the integration of the manual WhatsApp entry, autofill, data preservation, and the Principal dashboard UI update
</commit_message>
<xml_diff>
--- a/public/student_data.xlsx
+++ b/public/student_data.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\college-outpass-system\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0CA6BBE-B270-45B5-B4A1-1B78E32B3A43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72162A3C-D2E6-46D5-9539-2450BDEE4908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{7A0D0709-88B1-4457-A026-D8376796096F}"/>
   </bookViews>
   <sheets>
     <sheet name="student_data_sample" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">student_data_sample!$A$1:$G$2113</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -19699,7 +19702,7 @@
     <col min="1" max="2" width="30.140625" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.140625" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="30.140625" customWidth="1"/>
     <col min="6" max="6" width="30.140625" style="1" customWidth="1"/>
     <col min="7" max="7" width="29.85546875" bestFit="1" customWidth="1"/>
   </cols>
@@ -68304,6 +68307,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G2113" xr:uid="{0C039D9D-D42A-4C7C-86CD-5951C8D9D03A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>